<commit_message>
v2 pcb design progressing
</commit_message>
<xml_diff>
--- a/convention_badge_kicad/PCB_PART_SHEET.xlsx
+++ b/convention_badge_kicad/PCB_PART_SHEET.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bfcla\Programming_Projects\Embedded Systems\convention_pcb_badge\convention_badge_kicad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bfcla\Programming_Projects\Embedded_Systems\convention_pcb_badge\convention_badge_kicad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4EE6A772-E452-428E-92DC-6D9D189DE854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55B6D19-358C-45C2-83B3-9B23EF38C949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{254F5BF3-9C45-4EF7-80C1-1E1E6DA10C7F}"/>
+    <workbookView xWindow="8580" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{254F5BF3-9C45-4EF7-80C1-1E1E6DA10C7F}"/>
   </bookViews>
   <sheets>
     <sheet name="V1Parts" sheetId="1" r:id="rId1"/>
+    <sheet name="V2Parts" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
   <si>
     <t>Part Number</t>
   </si>
@@ -132,6 +133,18 @@
   </si>
   <si>
     <t>SW4</t>
+  </si>
+  <si>
+    <t>Part Number (JLCPCB)</t>
+  </si>
+  <si>
+    <t>Esp32C3</t>
+  </si>
+  <si>
+    <t>espressif</t>
+  </si>
+  <si>
+    <t>Surface Mount</t>
   </si>
 </sst>
 </file>
@@ -140,7 +153,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -205,9 +218,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -826,4 +839,72 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FAC52E-6AD2-4B1B-8B9B-70070407FE3E}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" customWidth="1"/>
+    <col min="7" max="7" width="24.21875" customWidth="1"/>
+    <col min="8" max="8" width="22.88671875" customWidth="1"/>
+    <col min="9" max="9" width="37.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <f>F2*G2</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>